<commit_message>
Korrektur bat var opex
</commit_message>
<xml_diff>
--- a/Ammoniak_Greenfield_Höchst/Datenbank.xlsx
+++ b/Ammoniak_Greenfield_Höchst/Datenbank.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01-Arbeit\06-FENES\09-P2X3\Ammoniak\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01-Arbeit\06-FENES\09-P2X3\FENES_P2X\Ammoniak_Greenfield_Höchst\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1486B266-CE9D-44CC-8142-F53FDDE59F8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8537F47-8298-4DE3-8ADF-36EF4CE0AC5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datenauswahl" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
     <author>Timon Geiß</author>
   </authors>
   <commentList>
-    <comment ref="E35" authorId="0" shapeId="0" xr:uid="{22946658-3822-4C9A-8007-CC034FA9B8AB}">
+    <comment ref="E34" authorId="0" shapeId="0" xr:uid="{22946658-3822-4C9A-8007-CC034FA9B8AB}">
       <text>
         <r>
           <rPr>
@@ -66,7 +66,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E36" authorId="0" shapeId="0" xr:uid="{426A9046-86EB-4AF9-8A2D-1FEFC7B6C4A3}">
+    <comment ref="E35" authorId="0" shapeId="0" xr:uid="{426A9046-86EB-4AF9-8A2D-1FEFC7B6C4A3}">
       <text>
         <r>
           <rPr>
@@ -90,7 +90,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E37" authorId="0" shapeId="0" xr:uid="{360FC6EE-8AD3-4EF7-B2BF-00DD1029DCAF}">
+    <comment ref="E36" authorId="0" shapeId="0" xr:uid="{360FC6EE-8AD3-4EF7-B2BF-00DD1029DCAF}">
       <text>
         <r>
           <rPr>
@@ -119,7 +119,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="295">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="294">
   <si>
     <t>PEM Elektrolyse</t>
   </si>
@@ -331,9 +331,6 @@
   </si>
   <si>
     <t>opex_fix_bat</t>
-  </si>
-  <si>
-    <t>opex_var_bat</t>
   </si>
   <si>
     <t>c_rate_bat</t>
@@ -1161,7 +1158,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="87">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -1223,9 +1220,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1268,32 +1265,23 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -1307,13 +1295,21 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1595,7 +1591,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.88671875" customWidth="1"/>
@@ -1613,7 +1609,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="12" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>2</v>
@@ -1634,7 +1630,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="58" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B2" s="68" t="s">
         <v>0</v>
@@ -1656,16 +1652,16 @@
       <c r="A3" s="59"/>
       <c r="B3" s="69"/>
       <c r="C3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E3" s="14">
         <v>50</v>
       </c>
       <c r="F3" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
@@ -1681,7 +1677,7 @@
         <v>1000</v>
       </c>
       <c r="F4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
@@ -1697,7 +1693,7 @@
         <v>0.03</v>
       </c>
       <c r="F5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
@@ -1738,26 +1734,26 @@
         <v>3</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E8" s="23">
         <v>1.8</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="59"/>
       <c r="B9" s="69"/>
       <c r="C9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E9" s="14">
         <v>285.39999999999998</v>
@@ -1779,7 +1775,7 @@
         <v>9070</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
@@ -1795,14 +1791,14 @@
         <v>0.05</v>
       </c>
       <c r="F11" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="59"/>
       <c r="B12" s="69"/>
       <c r="C12" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D12" t="s">
         <v>36</v>
@@ -1811,14 +1807,14 @@
         <v>0.17799999999999999</v>
       </c>
       <c r="F12" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="59"/>
       <c r="B13" s="69"/>
       <c r="C13" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D13" t="s">
         <v>37</v>
@@ -1827,7 +1823,7 @@
         <v>0.82199999999999995</v>
       </c>
       <c r="F13" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
@@ -1868,17 +1864,17 @@
         <v>4</v>
       </c>
       <c r="C16" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D16" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E16" s="14">
         <f>240/1000</f>
         <v>0.24</v>
       </c>
       <c r="F16" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
@@ -1894,7 +1890,7 @@
         <v>1990</v>
       </c>
       <c r="F17" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
@@ -1910,7 +1906,7 @@
         <v>0.05</v>
       </c>
       <c r="F18" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
@@ -1947,13 +1943,13 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="58" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B21" s="61" t="s">
         <v>5</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>45</v>
@@ -1962,7 +1958,7 @@
         <v>490</v>
       </c>
       <c r="F21" s="27" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
@@ -1978,7 +1974,7 @@
         <v>0.01</v>
       </c>
       <c r="F22" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
@@ -2010,7 +2006,7 @@
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="F24" s="13" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
@@ -2065,7 +2061,7 @@
       <c r="A28" s="59"/>
       <c r="B28" s="62"/>
       <c r="C28" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D28" t="s">
         <v>51</v>
@@ -2074,25 +2070,25 @@
         <v>0</v>
       </c>
       <c r="F28" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="59"/>
       <c r="B29" s="63" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E29" s="9">
         <v>1.6999999999999999E-3</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
@@ -2141,30 +2137,30 @@
         <v>2.5000000000000001E-2</v>
       </c>
       <c r="F32" s="52" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="59"/>
       <c r="B33" s="66"/>
       <c r="C33" s="52" t="s">
-        <v>20</v>
+        <v>47</v>
       </c>
       <c r="D33" s="52" t="s">
-        <v>70</v>
-      </c>
-      <c r="E33" s="53">
-        <v>0</v>
-      </c>
-      <c r="F33" s="55" t="s">
-        <v>21</v>
+        <v>71</v>
+      </c>
+      <c r="E33" s="54">
+        <v>0.93500000000000005</v>
+      </c>
+      <c r="F33" s="52" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="59"/>
       <c r="B34" s="66"/>
       <c r="C34" s="52" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D34" s="52" t="s">
         <v>72</v>
@@ -2180,396 +2176,380 @@
       <c r="A35" s="59"/>
       <c r="B35" s="66"/>
       <c r="C35" s="52" t="s">
-        <v>48</v>
+        <v>115</v>
       </c>
       <c r="D35" s="52" t="s">
-        <v>73</v>
-      </c>
-      <c r="E35" s="54">
-        <v>0.93500000000000005</v>
+        <v>70</v>
+      </c>
+      <c r="E35" s="53">
+        <v>0.25</v>
       </c>
       <c r="F35" s="52" t="s">
-        <v>24</v>
+        <v>116</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="59"/>
       <c r="B36" s="66"/>
       <c r="C36" s="52" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D36" s="52" t="s">
-        <v>71</v>
-      </c>
-      <c r="E36" s="53">
-        <v>0.25</v>
+        <v>73</v>
+      </c>
+      <c r="E36" s="54">
+        <v>0</v>
       </c>
       <c r="F36" s="52" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="59"/>
       <c r="B37" s="66"/>
       <c r="C37" s="52" t="s">
-        <v>115</v>
+        <v>15</v>
       </c>
       <c r="D37" s="52" t="s">
-        <v>74</v>
-      </c>
-      <c r="E37" s="54">
-        <v>0</v>
+        <v>66</v>
+      </c>
+      <c r="E37" s="55">
+        <v>15</v>
       </c>
       <c r="F37" s="52" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="59"/>
-      <c r="B38" s="66"/>
-      <c r="C38" s="52" t="s">
-        <v>15</v>
-      </c>
-      <c r="D38" s="52" t="s">
-        <v>66</v>
-      </c>
-      <c r="E38" s="56">
-        <v>15</v>
-      </c>
-      <c r="F38" s="52" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="60"/>
-      <c r="B39" s="67"/>
-      <c r="C39" s="15" t="s">
+    <row r="38" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="60"/>
+      <c r="B38" s="67"/>
+      <c r="C38" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="D39" s="15" t="s">
+      <c r="D38" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="E39" s="16">
+      <c r="E38" s="16">
         <v>0.1</v>
       </c>
-      <c r="F39" s="15" t="s">
+      <c r="F38" s="15" t="s">
         <v>24</v>
       </c>
     </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39" s="58" t="s">
+        <v>86</v>
+      </c>
+      <c r="B39" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E39" s="24">
+        <v>2000</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A40" s="58" t="s">
-        <v>87</v>
-      </c>
-      <c r="B40" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="E40" s="24">
-        <v>2000</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>21</v>
+      <c r="A40" s="59"/>
+      <c r="B40" s="63" t="s">
+        <v>6</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E40" s="9">
+        <v>0.99</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="59"/>
-      <c r="B41" s="63" t="s">
-        <v>6</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D41" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="E41" s="9">
-        <v>0.99</v>
-      </c>
-      <c r="F41" s="4" t="s">
-        <v>11</v>
+      <c r="B41" s="62"/>
+      <c r="C41" t="s">
+        <v>12</v>
+      </c>
+      <c r="D41" t="s">
+        <v>55</v>
+      </c>
+      <c r="E41" s="25">
+        <v>1100</v>
+      </c>
+      <c r="F41" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" s="59"/>
       <c r="B42" s="62"/>
       <c r="C42" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="D42" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E42" s="25">
-        <v>1100</v>
+        <v>17.84</v>
       </c>
       <c r="F42" t="s">
-        <v>14</v>
+        <v>118</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" s="59"/>
       <c r="B43" s="62"/>
       <c r="C43" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D43" t="s">
-        <v>56</v>
-      </c>
-      <c r="E43" s="25">
-        <v>17.84</v>
+        <v>57</v>
+      </c>
+      <c r="E43" s="14">
+        <v>0</v>
       </c>
       <c r="F43" t="s">
-        <v>119</v>
+        <v>21</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" s="59"/>
       <c r="B44" s="62"/>
       <c r="C44" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="D44" t="s">
-        <v>57</v>
-      </c>
-      <c r="E44" s="14">
-        <v>0</v>
+        <v>54</v>
+      </c>
+      <c r="E44" s="22">
+        <v>25</v>
       </c>
       <c r="F44" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" s="59"/>
       <c r="B45" s="62"/>
       <c r="C45" t="s">
-        <v>15</v>
+        <v>82</v>
       </c>
       <c r="D45" t="s">
-        <v>54</v>
-      </c>
-      <c r="E45" s="22">
-        <v>25</v>
+        <v>81</v>
+      </c>
+      <c r="E45" s="14">
+        <v>1000000</v>
       </c>
       <c r="F45" t="s">
-        <v>16</v>
+        <v>80</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" s="59"/>
-      <c r="B46" s="62"/>
-      <c r="C46" t="s">
-        <v>83</v>
-      </c>
-      <c r="D46" t="s">
-        <v>82</v>
-      </c>
-      <c r="E46" s="14">
-        <v>1000000</v>
-      </c>
-      <c r="F46" t="s">
-        <v>81</v>
+      <c r="B46" s="64"/>
+      <c r="C46" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D46" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="E46" s="10">
+        <v>5.2999999999999999E-2</v>
+      </c>
+      <c r="F46" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" s="59"/>
-      <c r="B47" s="64"/>
-      <c r="C47" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D47" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="E47" s="10">
-        <v>5.2999999999999999E-2</v>
-      </c>
-      <c r="F47" s="5" t="s">
+      <c r="B47" s="63" t="s">
+        <v>7</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E47" s="9">
+        <v>0.997</v>
+      </c>
+      <c r="F47" s="4" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" s="59"/>
-      <c r="B48" s="63" t="s">
-        <v>7</v>
-      </c>
-      <c r="C48" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D48" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="E48" s="9">
-        <v>0.997</v>
-      </c>
-      <c r="F48" s="4" t="s">
-        <v>24</v>
+      <c r="B48" s="62"/>
+      <c r="C48" t="s">
+        <v>12</v>
+      </c>
+      <c r="D48" t="s">
+        <v>60</v>
+      </c>
+      <c r="E48" s="25">
+        <v>1080</v>
+      </c>
+      <c r="F48" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" s="59"/>
       <c r="B49" s="62"/>
       <c r="C49" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="D49" t="s">
-        <v>60</v>
-      </c>
-      <c r="E49" s="25">
-        <v>1080</v>
-      </c>
-      <c r="F49" t="s">
-        <v>14</v>
+        <v>64</v>
+      </c>
+      <c r="E49" s="46">
+        <v>12.68</v>
+      </c>
+      <c r="F49" s="26" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="59"/>
       <c r="B50" s="62"/>
       <c r="C50" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D50" t="s">
-        <v>64</v>
-      </c>
-      <c r="E50" s="46">
-        <v>12.68</v>
-      </c>
-      <c r="F50" s="26" t="s">
-        <v>119</v>
+        <v>61</v>
+      </c>
+      <c r="E50" s="50">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="F50" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" s="59"/>
       <c r="B51" s="62"/>
       <c r="C51" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="D51" t="s">
-        <v>61</v>
-      </c>
-      <c r="E51" s="50">
-        <v>5.0000000000000001E-3</v>
+        <v>62</v>
+      </c>
+      <c r="E51" s="22">
+        <v>25</v>
       </c>
       <c r="F51" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" s="59"/>
       <c r="B52" s="62"/>
       <c r="C52" t="s">
-        <v>15</v>
+        <v>82</v>
       </c>
       <c r="D52" t="s">
-        <v>62</v>
-      </c>
-      <c r="E52" s="22">
-        <v>25</v>
+        <v>79</v>
+      </c>
+      <c r="E52" s="28">
+        <v>1000000</v>
       </c>
       <c r="F52" t="s">
-        <v>16</v>
+        <v>80</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A53" s="59"/>
-      <c r="B53" s="62"/>
-      <c r="C53" t="s">
-        <v>83</v>
-      </c>
-      <c r="D53" t="s">
-        <v>80</v>
-      </c>
-      <c r="E53" s="28">
-        <v>1000000</v>
-      </c>
-      <c r="F53" t="s">
-        <v>81</v>
+      <c r="A53" s="60"/>
+      <c r="B53" s="65"/>
+      <c r="C53" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="D53" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="E53" s="16">
+        <v>5.8000000000000003E-2</v>
+      </c>
+      <c r="F53" s="15" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A54" s="60"/>
-      <c r="B54" s="65"/>
-      <c r="C54" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="D54" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="E54" s="16">
-        <v>5.8000000000000003E-2</v>
-      </c>
-      <c r="F54" s="15" t="s">
-        <v>24</v>
+      <c r="A54" s="58" t="s">
+        <v>90</v>
+      </c>
+      <c r="B54" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="E54" s="3">
+        <v>-1E-4</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A55" s="58" t="s">
-        <v>91</v>
-      </c>
-      <c r="B55" s="17" t="s">
-        <v>88</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="D55" s="2" t="s">
+      <c r="A55" s="59"/>
+      <c r="B55" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="E55" s="3">
-        <v>-1E-4</v>
-      </c>
-      <c r="F55" s="2" t="s">
-        <v>21</v>
+      <c r="C55" s="19" t="s">
+        <v>95</v>
+      </c>
+      <c r="D55" s="19" t="s">
+        <v>97</v>
+      </c>
+      <c r="E55" s="20">
+        <v>-1.5</v>
+      </c>
+      <c r="F55" s="19" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A56" s="59"/>
-      <c r="B56" s="18" t="s">
+      <c r="A56" s="60"/>
+      <c r="B56" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="C56" s="19" t="s">
+      <c r="C56" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="D56" s="19" t="s">
+      <c r="D56" s="15" t="s">
         <v>98</v>
       </c>
-      <c r="E56" s="20">
-        <v>-1.5</v>
-      </c>
-      <c r="F56" s="19" t="s">
+      <c r="E56" s="16">
+        <v>-0.8</v>
+      </c>
+      <c r="F56" s="15" t="s">
         <v>100</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A57" s="60"/>
-      <c r="B57" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="C57" s="15" t="s">
-        <v>97</v>
-      </c>
-      <c r="D57" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="E57" s="16">
-        <v>-0.8</v>
-      </c>
-      <c r="F57" s="15" t="s">
-        <v>101</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="11">
     <mergeCell ref="A2:A20"/>
-    <mergeCell ref="A21:A39"/>
-    <mergeCell ref="A40:A54"/>
-    <mergeCell ref="A55:A57"/>
+    <mergeCell ref="A21:A38"/>
+    <mergeCell ref="A39:A53"/>
+    <mergeCell ref="A54:A56"/>
     <mergeCell ref="B21:B28"/>
-    <mergeCell ref="B41:B47"/>
-    <mergeCell ref="B48:B54"/>
-    <mergeCell ref="B29:B39"/>
+    <mergeCell ref="B40:B46"/>
+    <mergeCell ref="B47:B53"/>
+    <mergeCell ref="B29:B38"/>
     <mergeCell ref="B2:B7"/>
     <mergeCell ref="B8:B15"/>
     <mergeCell ref="B16:B20"/>
@@ -2596,7 +2576,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="30" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B1" s="31" t="s">
         <v>2</v>
@@ -2615,449 +2595,449 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="78" t="s">
-        <v>85</v>
-      </c>
-      <c r="B2" s="75" t="s">
+      <c r="A2" s="72" t="s">
+        <v>84</v>
+      </c>
+      <c r="B2" s="74" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="29" t="s">
+        <v>123</v>
+      </c>
+      <c r="D2" s="29" t="s">
         <v>124</v>
-      </c>
-      <c r="D2" s="29" t="s">
-        <v>125</v>
       </c>
       <c r="E2" s="33"/>
       <c r="F2" s="29" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="80"/>
-      <c r="B3" s="73"/>
+      <c r="A3" s="73"/>
+      <c r="B3" s="75"/>
       <c r="C3" s="13" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E3" s="34"/>
       <c r="F3" s="13" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="80"/>
-      <c r="B4" s="73"/>
+      <c r="A4" s="73"/>
+      <c r="B4" s="75"/>
       <c r="C4" s="13" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E4" s="35"/>
       <c r="F4" s="13" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="80"/>
-      <c r="B5" s="73"/>
+      <c r="A5" s="73"/>
+      <c r="B5" s="75"/>
       <c r="C5" s="13" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E5" s="36"/>
       <c r="F5" s="13" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="80"/>
-      <c r="B6" s="73"/>
+      <c r="A6" s="73"/>
+      <c r="B6" s="75"/>
       <c r="C6" s="13" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="E6" s="37"/>
       <c r="F6" s="13" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="80"/>
-      <c r="B7" s="73"/>
+      <c r="A7" s="73"/>
+      <c r="B7" s="75"/>
       <c r="C7" s="13" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E7" s="37"/>
       <c r="F7" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="80"/>
-      <c r="B8" s="73"/>
+      <c r="A8" s="73"/>
+      <c r="B8" s="75"/>
       <c r="C8" s="13" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E8" s="37"/>
       <c r="F8" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="80"/>
-      <c r="B9" s="73"/>
+      <c r="A9" s="73"/>
+      <c r="B9" s="75"/>
       <c r="C9" s="13" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="E9" s="37"/>
       <c r="F9" s="13" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="80"/>
-      <c r="B10" s="73"/>
+      <c r="A10" s="73"/>
+      <c r="B10" s="75"/>
       <c r="C10" s="13" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E10" s="37"/>
       <c r="F10" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="80"/>
-      <c r="B11" s="73"/>
+      <c r="A11" s="73"/>
+      <c r="B11" s="75"/>
       <c r="E11" s="36"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="80"/>
-      <c r="B12" s="72" t="s">
+      <c r="A12" s="73"/>
+      <c r="B12" s="76" t="s">
         <v>3</v>
       </c>
       <c r="C12" s="38" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D12" s="38" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E12" s="39"/>
       <c r="F12" s="38" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="80"/>
-      <c r="B13" s="73"/>
+      <c r="A13" s="73"/>
+      <c r="B13" s="75"/>
       <c r="C13" s="13" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E13" s="34"/>
       <c r="F13" s="13" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="80"/>
-      <c r="B14" s="73"/>
+      <c r="A14" s="73"/>
+      <c r="B14" s="75"/>
       <c r="C14" s="13" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E14" s="34"/>
       <c r="F14" s="34" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="80"/>
-      <c r="B15" s="73"/>
+      <c r="A15" s="73"/>
+      <c r="B15" s="75"/>
       <c r="C15" s="13" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E15" s="36"/>
       <c r="F15" s="13" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="80"/>
-      <c r="B16" s="73"/>
+      <c r="A16" s="73"/>
+      <c r="B16" s="75"/>
       <c r="C16" s="13" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E16" s="34"/>
       <c r="F16" s="13" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="80"/>
-      <c r="B17" s="73"/>
+      <c r="A17" s="73"/>
+      <c r="B17" s="75"/>
       <c r="C17" s="13" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E17" s="34"/>
       <c r="F17" s="13" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="80"/>
-      <c r="B18" s="73"/>
+      <c r="A18" s="73"/>
+      <c r="B18" s="75"/>
       <c r="C18" s="13" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E18" s="37"/>
       <c r="F18" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="80"/>
-      <c r="B19" s="73"/>
+      <c r="A19" s="73"/>
+      <c r="B19" s="75"/>
       <c r="C19" s="13" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E19" s="37"/>
       <c r="F19" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="80"/>
-      <c r="B20" s="73"/>
+      <c r="A20" s="73"/>
+      <c r="B20" s="75"/>
       <c r="C20" s="13" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D20" s="13" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E20" s="37"/>
       <c r="F20" s="13" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="80"/>
-      <c r="B21" s="73"/>
+      <c r="A21" s="73"/>
+      <c r="B21" s="75"/>
       <c r="C21" s="13" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E21" s="37"/>
       <c r="F21" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="80"/>
-      <c r="B22" s="76"/>
+      <c r="A22" s="73"/>
+      <c r="B22" s="77"/>
       <c r="C22" s="40"/>
       <c r="D22" s="40"/>
       <c r="E22" s="41"/>
       <c r="F22" s="40"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="80"/>
-      <c r="B23" s="81" t="s">
+      <c r="A23" s="73"/>
+      <c r="B23" s="78" t="s">
         <v>4</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E23" s="34"/>
       <c r="F23" s="13" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="80"/>
-      <c r="B24" s="81"/>
+      <c r="A24" s="73"/>
+      <c r="B24" s="78"/>
       <c r="C24" s="13" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E24" s="34"/>
       <c r="F24" s="13" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="80"/>
-      <c r="B25" s="81"/>
+      <c r="A25" s="73"/>
+      <c r="B25" s="78"/>
       <c r="C25" s="13" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E25" s="36"/>
       <c r="F25" s="13" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="80"/>
-      <c r="B26" s="81"/>
+      <c r="A26" s="73"/>
+      <c r="B26" s="78"/>
       <c r="C26" s="13" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D26" s="13" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E26" s="37"/>
       <c r="F26" s="13" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="80"/>
-      <c r="B27" s="81"/>
+      <c r="A27" s="73"/>
+      <c r="B27" s="78"/>
       <c r="C27" s="13" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D27" s="13" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E27" s="37"/>
       <c r="F27" s="13" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="80"/>
-      <c r="B28" s="81"/>
+      <c r="A28" s="73"/>
+      <c r="B28" s="78"/>
       <c r="C28" s="13" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D28" s="13" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E28" s="37"/>
       <c r="F28" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="80"/>
-      <c r="B29" s="81"/>
+      <c r="A29" s="73"/>
+      <c r="B29" s="78"/>
       <c r="C29" s="13" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D29" s="13" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E29" s="37"/>
       <c r="F29" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="80"/>
-      <c r="B30" s="81"/>
+      <c r="A30" s="73"/>
+      <c r="B30" s="78"/>
       <c r="C30" s="13" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D30" s="13" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="E30" s="36"/>
       <c r="F30" s="13" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="80"/>
-      <c r="B31" s="81"/>
+      <c r="A31" s="73"/>
+      <c r="B31" s="78"/>
       <c r="C31" s="13" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D31" s="13" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E31" s="36"/>
       <c r="F31" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="80"/>
-      <c r="B32" s="81"/>
+      <c r="A32" s="73"/>
+      <c r="B32" s="78"/>
       <c r="E32" s="36"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="78" t="s">
-        <v>86</v>
-      </c>
-      <c r="B33" s="83" t="s">
+      <c r="A33" s="72" t="s">
+        <v>85</v>
+      </c>
+      <c r="B33" s="80" t="s">
         <v>5</v>
       </c>
       <c r="C33" s="29" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D33" s="29" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E33" s="42"/>
       <c r="F33" s="48" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="80"/>
-      <c r="B34" s="81"/>
+      <c r="A34" s="73"/>
+      <c r="B34" s="78"/>
       <c r="C34" s="13" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D34" s="13" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E34" s="36"/>
       <c r="F34" s="49" t="s">
@@ -3065,1013 +3045,1006 @@
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="80"/>
-      <c r="B35" s="81"/>
+      <c r="A35" s="73"/>
+      <c r="B35" s="78"/>
       <c r="C35" s="13" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D35" s="13" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E35" s="37"/>
       <c r="F35" s="13" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="80"/>
-      <c r="B36" s="81"/>
+      <c r="A36" s="73"/>
+      <c r="B36" s="78"/>
       <c r="C36" s="13" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D36" s="13" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E36" s="36"/>
       <c r="F36" s="13" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" s="80"/>
-      <c r="B37" s="81"/>
+      <c r="A37" s="73"/>
+      <c r="B37" s="78"/>
       <c r="C37" s="13" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D37" s="13" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E37" s="36"/>
       <c r="F37" s="13" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="80"/>
-      <c r="B38" s="81"/>
+      <c r="A38" s="73"/>
+      <c r="B38" s="78"/>
       <c r="C38" s="13" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D38" s="13" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E38" s="36"/>
       <c r="F38" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39" s="80"/>
-      <c r="B39" s="81"/>
+      <c r="A39" s="73"/>
+      <c r="B39" s="78"/>
       <c r="C39" s="13" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D39" s="13" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E39" s="36"/>
       <c r="F39" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A40" s="80"/>
-      <c r="B40" s="81"/>
+      <c r="A40" s="73"/>
+      <c r="B40" s="78"/>
       <c r="C40" s="13" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D40" s="13" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E40" s="36"/>
       <c r="F40" s="13" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A41" s="80"/>
-      <c r="B41" s="81"/>
+      <c r="A41" s="73"/>
+      <c r="B41" s="78"/>
       <c r="C41" s="13" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D41" s="13" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E41" s="36"/>
       <c r="F41" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A42" s="80"/>
-      <c r="B42" s="81"/>
+      <c r="A42" s="73"/>
+      <c r="B42" s="78"/>
       <c r="E42" s="36"/>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A43" s="80"/>
-      <c r="B43" s="84" t="s">
+      <c r="A43" s="73"/>
+      <c r="B43" s="81" t="s">
         <v>8</v>
       </c>
       <c r="C43" s="38" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D43" s="38" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E43" s="43"/>
       <c r="F43" s="38" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A44" s="80"/>
-      <c r="B44" s="81"/>
+      <c r="A44" s="73"/>
+      <c r="B44" s="78"/>
       <c r="C44" s="13" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D44" s="13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E44" s="36"/>
       <c r="F44" s="13" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A45" s="80"/>
-      <c r="B45" s="73"/>
+      <c r="A45" s="73"/>
+      <c r="B45" s="75"/>
       <c r="C45" s="13" t="s">
+        <v>140</v>
+      </c>
+      <c r="D45" s="13" t="s">
         <v>141</v>
-      </c>
-      <c r="D45" s="13" t="s">
-        <v>142</v>
       </c>
       <c r="E45" s="34"/>
       <c r="F45" s="13" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A46" s="80"/>
-      <c r="B46" s="73"/>
+      <c r="A46" s="73"/>
+      <c r="B46" s="75"/>
       <c r="C46" s="13" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D46" s="13" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E46" s="34"/>
       <c r="F46" s="13" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A47" s="80"/>
-      <c r="B47" s="73"/>
+      <c r="A47" s="73"/>
+      <c r="B47" s="75"/>
       <c r="C47" s="13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D47" s="13" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E47" s="34"/>
       <c r="F47" s="13" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A48" s="80"/>
-      <c r="B48" s="73"/>
+      <c r="A48" s="73"/>
+      <c r="B48" s="75"/>
       <c r="C48" s="13" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D48" s="13" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E48" s="36"/>
       <c r="F48" s="13" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A49" s="80"/>
-      <c r="B49" s="73"/>
+      <c r="A49" s="73"/>
+      <c r="B49" s="75"/>
       <c r="C49" s="13" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D49" s="13" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E49" s="34"/>
       <c r="F49" s="13" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A50" s="80"/>
-      <c r="B50" s="73"/>
+      <c r="A50" s="73"/>
+      <c r="B50" s="75"/>
       <c r="C50" s="13" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D50" s="13" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E50" s="36"/>
       <c r="F50" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A51" s="80"/>
-      <c r="B51" s="73"/>
+      <c r="A51" s="73"/>
+      <c r="B51" s="75"/>
       <c r="C51" s="13" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D51" s="13" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E51" s="36"/>
       <c r="F51" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A52" s="80"/>
-      <c r="B52" s="73"/>
+      <c r="A52" s="73"/>
+      <c r="B52" s="75"/>
       <c r="C52" s="13" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D52" s="13" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E52" s="36"/>
       <c r="F52" s="13" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A53" s="80"/>
-      <c r="B53" s="73"/>
+      <c r="A53" s="73"/>
+      <c r="B53" s="75"/>
       <c r="C53" s="13" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D53" s="13" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E53" s="36"/>
       <c r="F53" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="54" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="82"/>
-      <c r="B54" s="74"/>
+      <c r="A54" s="79"/>
+      <c r="B54" s="82"/>
       <c r="C54" s="44"/>
       <c r="D54" s="44"/>
       <c r="E54" s="45"/>
       <c r="F54" s="44"/>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A55" s="78" t="s">
+      <c r="A55" s="72" t="s">
+        <v>86</v>
+      </c>
+      <c r="B55" s="74" t="s">
         <v>87</v>
       </c>
-      <c r="B55" s="75" t="s">
-        <v>88</v>
-      </c>
       <c r="C55" s="29" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D55" s="29" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E55" s="42"/>
       <c r="F55" s="29" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A56" s="80"/>
-      <c r="B56" s="73"/>
+      <c r="A56" s="73"/>
+      <c r="B56" s="75"/>
       <c r="C56" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D56" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E56" s="34"/>
       <c r="F56" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A57" s="80"/>
-      <c r="B57" s="76"/>
+      <c r="A57" s="73"/>
+      <c r="B57" s="77"/>
       <c r="E57" s="34"/>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A58" s="80"/>
-      <c r="B58" s="84" t="s">
+      <c r="A58" s="73"/>
+      <c r="B58" s="81" t="s">
         <v>6</v>
       </c>
       <c r="C58" s="38" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D58" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E58" s="43"/>
       <c r="F58" s="38" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A59" s="80"/>
-      <c r="B59" s="81"/>
+      <c r="A59" s="73"/>
+      <c r="B59" s="78"/>
       <c r="C59" s="13" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D59" s="13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E59" s="46"/>
       <c r="F59" s="13" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A60" s="80"/>
-      <c r="B60" s="81"/>
+      <c r="A60" s="73"/>
+      <c r="B60" s="78"/>
       <c r="C60" s="13" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D60" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E60" s="46"/>
       <c r="F60" s="13" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A61" s="80"/>
-      <c r="B61" s="81"/>
+      <c r="A61" s="73"/>
+      <c r="B61" s="78"/>
       <c r="C61" s="13" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D61" s="13" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E61" s="34"/>
       <c r="F61" s="13" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A62" s="80"/>
-      <c r="B62" s="81"/>
+      <c r="A62" s="73"/>
+      <c r="B62" s="78"/>
       <c r="C62" s="13" t="s">
+        <v>202</v>
+      </c>
+      <c r="D62" s="13" t="s">
         <v>203</v>
-      </c>
-      <c r="D62" s="13" t="s">
-        <v>204</v>
       </c>
       <c r="E62" s="37"/>
       <c r="F62" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A63" s="80"/>
-      <c r="B63" s="81"/>
+      <c r="A63" s="73"/>
+      <c r="B63" s="78"/>
       <c r="C63" s="13" t="s">
+        <v>210</v>
+      </c>
+      <c r="D63" s="13" t="s">
         <v>211</v>
-      </c>
-      <c r="D63" s="13" t="s">
-        <v>212</v>
       </c>
       <c r="E63" s="34"/>
       <c r="F63" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A64" s="80"/>
-      <c r="B64" s="81"/>
+      <c r="A64" s="73"/>
+      <c r="B64" s="78"/>
       <c r="C64" s="13" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D64" s="13" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="E64" s="34"/>
       <c r="F64" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A65" s="80"/>
-      <c r="B65" s="81"/>
+      <c r="A65" s="73"/>
+      <c r="B65" s="78"/>
       <c r="C65" s="13" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D65" s="13" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="E65" s="36"/>
       <c r="F65" s="13" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A66" s="80"/>
-      <c r="B66" s="81"/>
+      <c r="A66" s="73"/>
+      <c r="B66" s="78"/>
       <c r="C66" s="13" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D66" s="13" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E66" s="36"/>
       <c r="F66" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A67" s="80"/>
+      <c r="A67" s="73"/>
       <c r="B67" s="85"/>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A68" s="80"/>
-      <c r="B68" s="84" t="s">
+      <c r="A68" s="73"/>
+      <c r="B68" s="81" t="s">
         <v>7</v>
       </c>
       <c r="C68" s="38" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D68" s="38" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E68" s="43"/>
       <c r="F68" s="38" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A69" s="80"/>
-      <c r="B69" s="81"/>
+      <c r="A69" s="73"/>
+      <c r="B69" s="78"/>
       <c r="C69" s="13" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D69" s="13" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E69" s="46"/>
       <c r="F69" s="13" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A70" s="80"/>
-      <c r="B70" s="81"/>
+      <c r="A70" s="73"/>
+      <c r="B70" s="78"/>
       <c r="C70" s="13" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D70" s="13" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E70" s="46"/>
       <c r="F70" s="13" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A71" s="80"/>
-      <c r="B71" s="81"/>
+      <c r="A71" s="73"/>
+      <c r="B71" s="78"/>
       <c r="C71" s="13" t="s">
+        <v>184</v>
+      </c>
+      <c r="D71" s="13" t="s">
         <v>185</v>
-      </c>
-      <c r="D71" s="13" t="s">
-        <v>186</v>
       </c>
       <c r="E71" s="46"/>
       <c r="F71" s="13" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A72" s="80"/>
-      <c r="B72" s="81"/>
+      <c r="A72" s="73"/>
+      <c r="B72" s="78"/>
       <c r="C72" s="13" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D72" s="13" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E72" s="37"/>
       <c r="F72" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A73" s="80"/>
-      <c r="B73" s="81"/>
+      <c r="A73" s="73"/>
+      <c r="B73" s="78"/>
       <c r="C73" s="13" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D73" s="13" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E73" s="47"/>
       <c r="F73" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A74" s="80"/>
-      <c r="B74" s="81"/>
+      <c r="A74" s="73"/>
+      <c r="B74" s="78"/>
       <c r="C74" s="13" t="s">
+        <v>251</v>
+      </c>
+      <c r="D74" s="13" t="s">
         <v>252</v>
-      </c>
-      <c r="D74" s="13" t="s">
-        <v>253</v>
       </c>
       <c r="E74" s="47"/>
       <c r="F74" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A75" s="80"/>
-      <c r="B75" s="81"/>
+      <c r="A75" s="73"/>
+      <c r="B75" s="78"/>
       <c r="C75" s="13" t="s">
+        <v>216</v>
+      </c>
+      <c r="D75" s="13" t="s">
         <v>217</v>
-      </c>
-      <c r="D75" s="13" t="s">
-        <v>218</v>
       </c>
       <c r="E75" s="36"/>
       <c r="F75" s="13" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A76" s="80"/>
-      <c r="B76" s="81"/>
+      <c r="A76" s="73"/>
+      <c r="B76" s="78"/>
       <c r="C76" s="13" t="s">
+        <v>241</v>
+      </c>
+      <c r="D76" s="13" t="s">
         <v>242</v>
-      </c>
-      <c r="D76" s="13" t="s">
-        <v>243</v>
       </c>
       <c r="E76" s="36"/>
       <c r="F76" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="77" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A77" s="82"/>
+      <c r="A77" s="79"/>
       <c r="B77" s="86"/>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A78" s="78" t="s">
-        <v>91</v>
-      </c>
-      <c r="B78" s="75" t="s">
-        <v>88</v>
+      <c r="A78" s="72" t="s">
+        <v>90</v>
+      </c>
+      <c r="B78" s="74" t="s">
+        <v>87</v>
       </c>
       <c r="C78" s="29" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D78" s="29" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E78" s="33"/>
       <c r="F78" s="29" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A79" s="79"/>
-      <c r="B79" s="77"/>
-      <c r="C79" s="57" t="s">
-        <v>294</v>
-      </c>
-      <c r="D79" s="57" t="s">
+      <c r="A79" s="84"/>
+      <c r="B79" s="83"/>
+      <c r="C79" s="56" t="s">
         <v>293</v>
       </c>
-      <c r="E79" s="87"/>
-      <c r="F79" s="57" t="s">
+      <c r="D79" s="56" t="s">
+        <v>292</v>
+      </c>
+      <c r="E79" s="57"/>
+      <c r="F79" s="56" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A80" s="73"/>
+      <c r="B80" s="75"/>
+      <c r="C80" s="13" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A80" s="80"/>
-      <c r="B80" s="73"/>
-      <c r="C80" s="13" t="s">
-        <v>197</v>
-      </c>
       <c r="D80" s="13" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E80" s="36"/>
       <c r="F80" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A81" s="80"/>
-      <c r="B81" s="76"/>
+      <c r="A81" s="73"/>
+      <c r="B81" s="77"/>
       <c r="E81" s="36"/>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A82" s="80"/>
-      <c r="B82" s="72" t="s">
-        <v>94</v>
+      <c r="A82" s="73"/>
+      <c r="B82" s="76" t="s">
+        <v>93</v>
       </c>
       <c r="C82" s="38" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D82" s="38" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E82" s="43"/>
       <c r="F82" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A83" s="80"/>
-      <c r="B83" s="73"/>
+      <c r="A83" s="73"/>
+      <c r="B83" s="75"/>
       <c r="C83" s="13" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D83" s="13" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E83" s="36"/>
       <c r="F83" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A84" s="80"/>
-      <c r="B84" s="76"/>
+      <c r="A84" s="73"/>
+      <c r="B84" s="77"/>
       <c r="C84" s="40"/>
       <c r="D84" s="40"/>
       <c r="E84" s="41"/>
       <c r="F84" s="40"/>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A85" s="80"/>
-      <c r="B85" s="72" t="s">
-        <v>95</v>
+      <c r="A85" s="73"/>
+      <c r="B85" s="76" t="s">
+        <v>94</v>
       </c>
       <c r="C85" s="13" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D85" s="13" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E85" s="36"/>
       <c r="F85" s="13" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A86" s="80"/>
-      <c r="B86" s="73"/>
+      <c r="A86" s="73"/>
+      <c r="B86" s="75"/>
       <c r="C86" s="13" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D86" s="13" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E86" s="36"/>
       <c r="F86" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="87" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A87" s="82"/>
-      <c r="B87" s="74"/>
+      <c r="A87" s="79"/>
+      <c r="B87" s="82"/>
       <c r="C87" s="44"/>
       <c r="D87" s="44"/>
       <c r="E87" s="45"/>
       <c r="F87" s="44"/>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A88" s="78" t="s">
-        <v>213</v>
-      </c>
-      <c r="B88" s="75" t="s">
+      <c r="A88" s="72" t="s">
+        <v>212</v>
+      </c>
+      <c r="B88" s="74" t="s">
         <v>15</v>
       </c>
       <c r="C88" s="29" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D88" s="29" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E88" s="29"/>
       <c r="F88" s="29" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A89" s="79"/>
-      <c r="B89" s="73"/>
+      <c r="A89" s="84"/>
+      <c r="B89" s="75"/>
       <c r="C89" s="13" t="s">
+        <v>225</v>
+      </c>
+      <c r="D89" s="13" t="s">
         <v>226</v>
       </c>
-      <c r="D89" s="13" t="s">
-        <v>227</v>
-      </c>
       <c r="F89" s="13" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A90" s="79"/>
-      <c r="B90" s="76"/>
+      <c r="A90" s="84"/>
+      <c r="B90" s="77"/>
       <c r="C90" s="40"/>
       <c r="D90" s="40"/>
       <c r="E90" s="40"/>
       <c r="F90" s="40"/>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A91" s="79"/>
-      <c r="B91" s="72" t="s">
-        <v>236</v>
+      <c r="A91" s="84"/>
+      <c r="B91" s="76" t="s">
+        <v>235</v>
       </c>
       <c r="C91" s="13" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D91" s="13" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F91" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A92" s="79"/>
-      <c r="B92" s="73"/>
+      <c r="A92" s="84"/>
+      <c r="B92" s="75"/>
       <c r="C92" s="13" t="s">
+        <v>233</v>
+      </c>
+      <c r="D92" s="13" t="s">
+        <v>227</v>
+      </c>
+      <c r="F92" s="13" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A93" s="84"/>
+      <c r="B93" s="75"/>
+      <c r="C93" s="13" t="s">
+        <v>229</v>
+      </c>
+      <c r="D93" s="13" t="s">
+        <v>228</v>
+      </c>
+      <c r="F93" s="13" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A94" s="84"/>
+      <c r="B94" s="75"/>
+      <c r="C94" s="13" t="s">
+        <v>231</v>
+      </c>
+      <c r="D94" s="13" t="s">
+        <v>230</v>
+      </c>
+      <c r="F94" s="13" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A95" s="84"/>
+      <c r="B95" s="75"/>
+      <c r="C95" s="13" t="s">
         <v>234</v>
       </c>
-      <c r="D92" s="13" t="s">
-        <v>228</v>
-      </c>
-      <c r="F92" s="13" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A93" s="79"/>
-      <c r="B93" s="73"/>
-      <c r="C93" s="13" t="s">
-        <v>230</v>
-      </c>
-      <c r="D93" s="13" t="s">
-        <v>229</v>
-      </c>
-      <c r="F93" s="13" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A94" s="79"/>
-      <c r="B94" s="73"/>
-      <c r="C94" s="13" t="s">
+      <c r="D95" s="13" t="s">
         <v>232</v>
       </c>
-      <c r="D94" s="13" t="s">
-        <v>231</v>
-      </c>
-      <c r="F94" s="13" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A95" s="79"/>
-      <c r="B95" s="73"/>
-      <c r="C95" s="13" t="s">
-        <v>235</v>
-      </c>
-      <c r="D95" s="13" t="s">
-        <v>233</v>
-      </c>
       <c r="F95" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A96" s="79"/>
-      <c r="B96" s="73"/>
+      <c r="A96" s="84"/>
+      <c r="B96" s="75"/>
       <c r="C96" s="13" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D96" s="13" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F96" s="13" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A97" s="79"/>
-      <c r="B97" s="72" t="s">
+      <c r="A97" s="84"/>
+      <c r="B97" s="76" t="s">
+        <v>265</v>
+      </c>
+      <c r="C97" s="38" t="s">
+        <v>260</v>
+      </c>
+      <c r="D97" s="38" t="s">
         <v>266</v>
-      </c>
-      <c r="C97" s="38" t="s">
-        <v>261</v>
-      </c>
-      <c r="D97" s="38" t="s">
-        <v>267</v>
       </c>
       <c r="E97" s="38"/>
       <c r="F97" s="38" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A98" s="84"/>
+      <c r="B98" s="83"/>
+      <c r="C98" s="56" t="s">
+        <v>261</v>
+      </c>
+      <c r="D98" s="56" t="s">
+        <v>269</v>
+      </c>
+      <c r="E98" s="56"/>
+      <c r="F98" s="56" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A99" s="84"/>
+      <c r="B99" s="83"/>
+      <c r="C99" s="56" t="s">
+        <v>276</v>
+      </c>
+      <c r="D99" s="56" t="s">
+        <v>275</v>
+      </c>
+      <c r="E99" s="56"/>
+      <c r="F99" s="56" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A100" s="84"/>
+      <c r="B100" s="83"/>
+      <c r="C100" s="56" t="s">
+        <v>262</v>
+      </c>
+      <c r="D100" s="56" t="s">
         <v>268</v>
       </c>
-    </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A98" s="79"/>
-      <c r="B98" s="77"/>
-      <c r="C98" s="57" t="s">
-        <v>262</v>
-      </c>
-      <c r="D98" s="57" t="s">
+      <c r="E100" s="56"/>
+      <c r="F100" s="56" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A101" s="84"/>
+      <c r="B101" s="83"/>
+      <c r="C101" s="56" t="s">
+        <v>278</v>
+      </c>
+      <c r="D101" s="56" t="s">
+        <v>277</v>
+      </c>
+      <c r="E101" s="56"/>
+      <c r="F101" s="56" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A102" s="84"/>
+      <c r="B102" s="83"/>
+      <c r="C102" s="56" t="s">
+        <v>282</v>
+      </c>
+      <c r="D102" s="56" t="s">
         <v>270</v>
       </c>
-      <c r="E98" s="57"/>
-      <c r="F98" s="57" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A99" s="79"/>
-      <c r="B99" s="77"/>
-      <c r="C99" s="57" t="s">
-        <v>277</v>
-      </c>
-      <c r="D99" s="57" t="s">
-        <v>276</v>
-      </c>
-      <c r="E99" s="57"/>
-      <c r="F99" s="57" t="s">
+      <c r="E102" s="56"/>
+      <c r="F102" s="56" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A103" s="84"/>
+      <c r="B103" s="83"/>
+      <c r="C103" s="56" t="s">
+        <v>259</v>
+      </c>
+      <c r="D103" s="13" t="s">
         <v>281</v>
       </c>
-    </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A100" s="79"/>
-      <c r="B100" s="77"/>
-      <c r="C100" s="57" t="s">
+      <c r="E103" s="56"/>
+      <c r="F103" s="56" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A104" s="84"/>
+      <c r="B104" s="83"/>
+      <c r="C104" s="56" t="s">
         <v>263</v>
       </c>
-      <c r="D100" s="57" t="s">
-        <v>269</v>
-      </c>
-      <c r="E100" s="57"/>
-      <c r="F100" s="57" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A101" s="79"/>
-      <c r="B101" s="77"/>
-      <c r="C101" s="57" t="s">
-        <v>279</v>
-      </c>
-      <c r="D101" s="57" t="s">
-        <v>278</v>
-      </c>
-      <c r="E101" s="57"/>
-      <c r="F101" s="57" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A102" s="79"/>
-      <c r="B102" s="77"/>
-      <c r="C102" s="57" t="s">
+      <c r="D104" s="56" t="s">
+        <v>272</v>
+      </c>
+      <c r="E104" s="56"/>
+      <c r="F104" s="13" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A105" s="84"/>
+      <c r="B105" s="83"/>
+      <c r="C105" s="56" t="s">
+        <v>264</v>
+      </c>
+      <c r="D105" s="56" t="s">
+        <v>273</v>
+      </c>
+      <c r="E105" s="56"/>
+      <c r="F105" s="56" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A106" s="84"/>
+      <c r="B106" s="76" t="s">
         <v>283</v>
       </c>
-      <c r="D102" s="57" t="s">
-        <v>271</v>
-      </c>
-      <c r="E102" s="57"/>
-      <c r="F102" s="57" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A103" s="79"/>
-      <c r="B103" s="77"/>
-      <c r="C103" s="57" t="s">
-        <v>260</v>
-      </c>
-      <c r="D103" s="13" t="s">
-        <v>282</v>
-      </c>
-      <c r="E103" s="57"/>
-      <c r="F103" s="57" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A104" s="79"/>
-      <c r="B104" s="77"/>
-      <c r="C104" s="57" t="s">
-        <v>264</v>
-      </c>
-      <c r="D104" s="57" t="s">
-        <v>273</v>
-      </c>
-      <c r="E104" s="57"/>
-      <c r="F104" s="13" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A105" s="79"/>
-      <c r="B105" s="77"/>
-      <c r="C105" s="57" t="s">
-        <v>265</v>
-      </c>
-      <c r="D105" s="57" t="s">
-        <v>274</v>
-      </c>
-      <c r="E105" s="57"/>
-      <c r="F105" s="57" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A106" s="79"/>
-      <c r="B106" s="72" t="s">
+      <c r="C106" s="38" t="s">
+        <v>285</v>
+      </c>
+      <c r="D106" s="38" t="s">
         <v>284</v>
-      </c>
-      <c r="C106" s="38" t="s">
-        <v>286</v>
-      </c>
-      <c r="D106" s="38" t="s">
-        <v>285</v>
       </c>
       <c r="E106" s="38"/>
       <c r="F106" s="38" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A107" s="79"/>
-      <c r="B107" s="77"/>
-      <c r="C107" s="57" t="s">
+      <c r="A107" s="84"/>
+      <c r="B107" s="83"/>
+      <c r="C107" s="56" t="s">
+        <v>286</v>
+      </c>
+      <c r="D107" s="56" t="s">
         <v>287</v>
       </c>
-      <c r="D107" s="57" t="s">
+      <c r="E107" s="56"/>
+      <c r="F107" s="56" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A108" s="84"/>
+      <c r="B108" s="83"/>
+      <c r="C108" s="56" t="s">
         <v>288</v>
       </c>
-      <c r="E107" s="57"/>
-      <c r="F107" s="57" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A108" s="79"/>
-      <c r="B108" s="77"/>
-      <c r="C108" s="57" t="s">
+      <c r="D108" s="56" t="s">
+        <v>290</v>
+      </c>
+      <c r="E108" s="56"/>
+      <c r="F108" s="56" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A109" s="84"/>
+      <c r="B109" s="83"/>
+      <c r="C109" s="13" t="s">
         <v>289</v>
       </c>
-      <c r="D108" s="57" t="s">
+      <c r="D109" s="13" t="s">
         <v>291</v>
       </c>
-      <c r="E108" s="57"/>
-      <c r="F108" s="57" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A109" s="79"/>
-      <c r="B109" s="77"/>
-      <c r="C109" s="13" t="s">
-        <v>290</v>
-      </c>
-      <c r="D109" s="13" t="s">
-        <v>292</v>
-      </c>
       <c r="F109" s="13" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="A2:A32"/>
-    <mergeCell ref="B2:B11"/>
-    <mergeCell ref="B12:B22"/>
-    <mergeCell ref="B23:B32"/>
-    <mergeCell ref="A33:A54"/>
-    <mergeCell ref="B33:B42"/>
-    <mergeCell ref="B43:B54"/>
     <mergeCell ref="B85:B87"/>
     <mergeCell ref="B55:B57"/>
     <mergeCell ref="B91:B96"/>
@@ -4085,6 +4058,13 @@
     <mergeCell ref="A78:A87"/>
     <mergeCell ref="B78:B81"/>
     <mergeCell ref="B82:B84"/>
+    <mergeCell ref="A2:A32"/>
+    <mergeCell ref="B2:B11"/>
+    <mergeCell ref="B12:B22"/>
+    <mergeCell ref="B23:B32"/>
+    <mergeCell ref="A33:A54"/>
+    <mergeCell ref="B33:B42"/>
+    <mergeCell ref="B43:B54"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>